<commit_message>
Edited the jupiter file to track materials sent to landfill by editing F_3_0 to F_3_9, adding the correspioding entry in the ConfigT6 File, and adding the landfill rate parameter file
</commit_message>
<xml_diff>
--- a/docs/Files/JV_T6_plusLF/ODYM_Config_Tutorial6.xlsx
+++ b/docs/Files/JV_T6_plusLF/ODYM_Config_Tutorial6.xlsx
@@ -1,26 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spauliuk.AD\FILES\ARBEIT\PROJECTS\ODYM-RECC\ODYM_Model\docs\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\JV_T6_plusLF\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D58C1E-6890-48A2-BBD2-CB52851DA3EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21158" windowHeight="10320" tabRatio="844" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="5" r:id="rId1"/>
     <sheet name="Setting_Tutorial6" sheetId="6" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="136">
   <si>
     <t>Description</t>
   </si>
@@ -413,12 +427,27 @@
   </si>
   <si>
     <t>Scenario analysis of dispersion of steel into different applications.</t>
+  </si>
+  <si>
+    <t>Landfill</t>
+  </si>
+  <si>
+    <t>ODYM_P9_EoLLandfillRate</t>
+  </si>
+  <si>
+    <t>EoL landfilling rate of steel scrap from products</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e6</t>
+  </si>
+  <si>
+    <t>Not part of original T6, nor is P9 in model parameters</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -614,7 +643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -622,54 +651,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -700,21 +716,16 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -991,194 +1002,180 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.53125" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B1" s="36" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="16" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="8"/>
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="6"/>
+      <c r="B2" s="8" t="s">
         <v>40</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="20"/>
-    </row>
-    <row r="3" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="8"/>
-      <c r="B3" s="12"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="6"/>
+      <c r="B3" s="8"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="5"/>
-      <c r="G3" s="20"/>
-    </row>
-    <row r="4" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="8"/>
-      <c r="B4" s="13" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6"/>
+      <c r="B4" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G4" s="44"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" s="8"/>
-      <c r="B5" s="13" t="s">
+      <c r="G4" s="35"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="6"/>
+      <c r="B5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="5" t="str">
+      <c r="C5" s="2"/>
+      <c r="D5" t="str">
         <f>E5&amp;D4</f>
         <v>Setting_Tutorial6</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" s="8"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A7" s="8"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" s="8"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" s="10"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" s="15"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A11" s="15"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A12" s="15"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" s="15"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A14" s="15"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" s="15"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" s="15"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A17" s="15"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" s="15"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19" s="15"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" s="15"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21" s="15"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A22" s="15"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A23" s="15"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24" s="15"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A25" s="10"/>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="6"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="10"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="12"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="10"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="10"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="10"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="10"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="10"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="10"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="10"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="10"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="10"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="10"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="10"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="10"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A26" s="10"/>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="6"/>
       <c r="B26" s="1"/>
       <c r="C26" s="2"/>
     </row>
@@ -1189,199 +1186,169 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:K59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="B2:J61"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="4.86328125" customWidth="1"/>
+    <col min="2" max="2" width="4.88671875" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="44.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.6640625" customWidth="1"/>
-    <col min="6" max="6" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B2" s="25" t="s">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="27"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C3" s="30" t="s">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="20"/>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.45">
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="20"/>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="D7" s="11"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="20"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B8" s="25" t="s">
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="D7" s="7"/>
+      <c r="J7" s="13"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B8" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="20"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C9" s="30" t="s">
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="20"/>
+      <c r="J8" s="13"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="20"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="J9" s="13"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="20"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="J10" s="13"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="I11" s="20"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="20"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="J11" s="13"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="I12" s="20"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="20"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="I13" s="20"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="20"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B14" s="25" t="s">
+      <c r="J12" s="13"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="J13" s="17"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B14" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26" t="s">
+      <c r="C14" s="19"/>
+      <c r="D14" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C15" s="31" t="s">
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="20"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="30" t="s">
+      <c r="E15" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="30" t="s">
+      <c r="F15" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="30" t="s">
+      <c r="G15" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="29" t="s">
+      <c r="H15" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="43" t="s">
+      <c r="I15" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="J15" s="35" t="s">
+      <c r="J15" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="20"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C16" s="32" t="s">
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="25" t="s">
         <v>11</v>
       </c>
       <c r="D16" t="s">
@@ -1393,20 +1360,18 @@
       <c r="F16" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" t="s">
         <v>129</v>
       </c>
-      <c r="H16" s="28" t="s">
+      <c r="H16" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I16" s="20" t="s">
+      <c r="I16" t="s">
         <v>68</v>
       </c>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C17" s="32" t="s">
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C17" s="25" t="s">
         <v>76</v>
       </c>
       <c r="D17" t="s">
@@ -1418,20 +1383,18 @@
       <c r="F17" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" t="s">
         <v>129</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="H17" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="I17" s="20" t="s">
+      <c r="I17" t="s">
         <v>79</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C18" s="32" t="s">
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C18" s="25" t="s">
         <v>15</v>
       </c>
       <c r="D18" t="s">
@@ -1443,20 +1406,18 @@
       <c r="F18" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="G18" t="s">
         <v>128</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="I18" t="s">
         <v>69</v>
       </c>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C19" s="32" t="s">
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C19" s="25" t="s">
         <v>16</v>
       </c>
       <c r="D19" t="s">
@@ -1471,17 +1432,15 @@
       <c r="G19" t="s">
         <v>91</v>
       </c>
-      <c r="H19" s="28">
+      <c r="H19" s="21">
         <v>1</v>
       </c>
-      <c r="I19" s="20" t="s">
+      <c r="I19" t="s">
         <v>71</v>
       </c>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C20" s="32" t="s">
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C20" s="25" t="s">
         <v>82</v>
       </c>
       <c r="D20" t="s">
@@ -1496,17 +1455,15 @@
       <c r="G20" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="28" t="s">
+      <c r="H20" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="I20" s="20" t="s">
+      <c r="I20" t="s">
         <v>85</v>
       </c>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C21" s="32" t="s">
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C21" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D21" t="s">
@@ -1521,15 +1478,15 @@
       <c r="G21" t="s">
         <v>91</v>
       </c>
-      <c r="H21" s="28" t="s">
+      <c r="H21" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="I21" s="20" t="s">
+      <c r="I21" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C22" s="32" t="s">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C22" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D22" t="s">
@@ -1544,15 +1501,15 @@
       <c r="G22" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="28" t="s">
+      <c r="H22" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="20" t="s">
+      <c r="I22" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C23" s="32" t="s">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C23" s="25" t="s">
         <v>14</v>
       </c>
       <c r="D23" t="s">
@@ -1567,15 +1524,15 @@
       <c r="G23" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="28" t="s">
+      <c r="H23" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="I23" s="20" t="s">
+      <c r="I23" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C24" s="47" t="s">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C24" s="21" t="s">
         <v>94</v>
       </c>
       <c r="D24" t="s">
@@ -1590,42 +1547,42 @@
       <c r="G24" t="s">
         <v>91</v>
       </c>
-      <c r="H24" s="28" t="s">
+      <c r="H24" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="I24" s="20" t="s">
+      <c r="I24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B26" s="25" t="s">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="27"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C27" s="33" t="s">
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="20"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C27" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="E27" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="F27" s="30" t="s">
+      <c r="F27" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37"/>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C28" s="38">
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C28" s="31">
         <v>0</v>
       </c>
       <c r="D28" t="s">
@@ -1635,8 +1592,8 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C29" s="38">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C29" s="31">
         <v>1</v>
       </c>
       <c r="D29" t="s">
@@ -1646,8 +1603,8 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C30" s="34">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C30" s="27">
         <v>2</v>
       </c>
       <c r="D30" t="s">
@@ -1657,8 +1614,8 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C31" s="34">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C31" s="27">
         <v>3</v>
       </c>
       <c r="D31" t="s">
@@ -1668,8 +1625,8 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="C32" s="38">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C32" s="31">
         <v>4</v>
       </c>
       <c r="D32" t="s">
@@ -1679,8 +1636,8 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C33" s="34">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C33" s="27">
         <v>5</v>
       </c>
       <c r="D33" t="s">
@@ -1690,8 +1647,8 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C34" s="38">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C34" s="31">
         <v>6</v>
       </c>
       <c r="D34" t="s">
@@ -1701,8 +1658,8 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C35" s="34">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C35" s="27">
         <v>7</v>
       </c>
       <c r="D35" t="s">
@@ -1712,8 +1669,8 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C36" s="38">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C36" s="31">
         <v>8</v>
       </c>
       <c r="D36" t="s">
@@ -1723,246 +1680,283 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B38" s="25" t="s">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C37" s="31">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F37" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B39" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="27"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C39" s="33" t="s">
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="20"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C40" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="30" t="s">
+      <c r="D40" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E39" s="30" t="s">
+      <c r="E40" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="F39" s="30" t="s">
+      <c r="F40" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="G39" s="30" t="s">
+      <c r="G40" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="H39" s="30" t="s">
+      <c r="H40" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I39" s="45" t="s">
+      <c r="I40" s="36" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C40" t="s">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
         <v>101</v>
       </c>
-      <c r="D40" s="48" t="s">
+      <c r="D41" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E40" s="20" t="s">
+      <c r="E41" t="s">
         <v>100</v>
       </c>
-      <c r="F40" s="20" t="s">
+      <c r="F41" t="s">
         <v>64</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G41" t="s">
         <v>31</v>
-      </c>
-      <c r="H40" t="s">
-        <v>31</v>
-      </c>
-      <c r="I40" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C41" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41" t="s">
-        <v>107</v>
-      </c>
-      <c r="E41" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="F41" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="G41" s="20" t="s">
-        <v>81</v>
       </c>
       <c r="H41" t="s">
         <v>31</v>
       </c>
       <c r="I41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C42" s="34" t="s">
-        <v>105</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C42" s="27" t="s">
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>108</v>
-      </c>
-      <c r="E42" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="E42" t="s">
         <v>100</v>
       </c>
-      <c r="F42" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="G42" s="20" t="s">
+      <c r="F42" t="s">
+        <v>110</v>
+      </c>
+      <c r="G42" t="s">
         <v>81</v>
       </c>
       <c r="H42" t="s">
         <v>31</v>
       </c>
-      <c r="I42" s="46" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C43" s="34" t="s">
-        <v>113</v>
+      <c r="I42" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C43" s="27" t="s">
+        <v>105</v>
       </c>
       <c r="D43" t="s">
-        <v>114</v>
-      </c>
-      <c r="E43" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E43" t="s">
         <v>100</v>
       </c>
-      <c r="F43" s="20" t="s">
+      <c r="F43" t="s">
         <v>109</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="G43" t="s">
         <v>81</v>
       </c>
       <c r="H43" t="s">
         <v>31</v>
       </c>
-      <c r="I43" s="46" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C44" s="34" t="s">
-        <v>116</v>
+      <c r="I43" s="37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C44" s="27" t="s">
+        <v>113</v>
       </c>
       <c r="D44" t="s">
-        <v>119</v>
-      </c>
-      <c r="E44" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="E44" t="s">
         <v>100</v>
       </c>
-      <c r="F44" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="G44" s="20" t="s">
-        <v>87</v>
+      <c r="F44" t="s">
+        <v>109</v>
+      </c>
+      <c r="G44" t="s">
+        <v>81</v>
       </c>
       <c r="H44" t="s">
         <v>31</v>
       </c>
-      <c r="I44" s="46" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C45" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="E45" s="20" t="s">
+      <c r="I44" s="37" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C45" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="D45" t="s">
+        <v>119</v>
+      </c>
+      <c r="E45" t="s">
         <v>100</v>
       </c>
-      <c r="F45" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="G45" s="20" t="s">
+      <c r="F45" t="s">
+        <v>118</v>
+      </c>
+      <c r="G45" t="s">
         <v>87</v>
       </c>
       <c r="H45" t="s">
         <v>31</v>
       </c>
-      <c r="I45" s="46" t="s">
+      <c r="I45" s="37" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C46" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="E46" t="s">
+        <v>100</v>
+      </c>
+      <c r="F46" t="s">
+        <v>121</v>
+      </c>
+      <c r="G46" t="s">
+        <v>87</v>
+      </c>
+      <c r="H46" t="s">
+        <v>31</v>
+      </c>
+      <c r="I46" s="37" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C46" s="34"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B47" s="25" t="s">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C47" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="D47" t="s">
+        <v>133</v>
+      </c>
+      <c r="E47" t="s">
+        <v>100</v>
+      </c>
+      <c r="F47" t="s">
+        <v>109</v>
+      </c>
+      <c r="G47" t="s">
+        <v>81</v>
+      </c>
+      <c r="H47" t="s">
+        <v>31</v>
+      </c>
+      <c r="I47" s="37" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C48" s="27"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B49" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="27"/>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C48" t="s">
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="20"/>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C50" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="C49" s="34" t="s">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C51" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="D49" s="40" t="s">
+      <c r="D51" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E51" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="D50" s="40"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="D51" s="40"/>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="D52" s="40"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="D53" s="40"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="D54" s="40"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B56" s="25" t="s">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D52" s="33"/>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D53" s="33"/>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D54" s="33"/>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D55" s="33"/>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D56" s="33"/>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B58" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
-      <c r="G56" s="26"/>
-      <c r="H56" s="27"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="C57" t="s">
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="20"/>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C59" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B59" s="25" t="s">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B61" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C59" s="26"/>
-      <c r="D59" s="26"/>
-      <c r="E59" s="26"/>
-      <c r="F59" s="26"/>
-      <c r="G59" s="26"/>
-      <c r="H59" s="27"/>
+      <c r="C61" s="19"/>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
+      <c r="F61" s="19"/>
+      <c r="G61" s="19"/>
+      <c r="H61" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>